<commit_message>
all things are done
</commit_message>
<xml_diff>
--- a/public/CandidatesForAssessment.xlsx
+++ b/public/CandidatesForAssessment.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hr\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\assessment_dashboard\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ECF5250-F14D-413A-B709-44D505E8A786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7500"/>
+    <workbookView xWindow="4065" yWindow="4065" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,15 +33,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>email</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>phone_number</t>
+  </si>
+  <si>
+    <t>college_name</t>
+  </si>
+  <si>
+    <t>year_of_passing</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="3">
     <font>
       <sz val="11"/>
@@ -296,7 +309,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="16"/>
       <tableStyleElement type="headerRow" dxfId="15"/>
       <tableStyleElement type="totalRow" dxfId="14"/>
@@ -305,7 +318,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="11"/>
       <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
       <tableStyleElement type="headerRow" dxfId="9"/>
       <tableStyleElement type="totalRow" dxfId="8"/>
       <tableStyleElement type="firstRowStripe" dxfId="7"/>
@@ -586,22 +599,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="29.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
     </row>
-    <row r="2" spans="1:1">
+    <row r="2" spans="1:5">
       <c r="A2" s="2"/>
     </row>
-    <row r="3" spans="1:1">
+    <row r="3" spans="1:5">
       <c r="A3" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
edit profile,single candidate, download mail students,submission time,etc
</commit_message>
<xml_diff>
--- a/public/CandidatesForAssessment.xlsx
+++ b/public/CandidatesForAssessment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\assessment_dashboard\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ECF5250-F14D-413A-B709-44D505E8A786}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D10028AF-CE57-4FAB-8A7D-CB060EA8CE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4065" yWindow="4065" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,8 +24,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -33,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
   <si>
     <t>email</t>
   </si>
@@ -48,6 +46,12 @@
   </si>
   <si>
     <t>year_of_passing</t>
+  </si>
+  <si>
+    <t>demo@example.com</t>
+  </si>
+  <si>
+    <t>demo</t>
   </si>
 </sst>
 </file>
@@ -600,10 +604,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="29.85546875" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -624,12 +629,26 @@
       </c>
     </row>
     <row r="2" spans="1:5">
-      <c r="A2" s="2"/>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" s="2"/>
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <v>1234567890</v>
+      </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2">
+        <v>1999</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" xr:uid="{72044284-2439-4E38-8CF9-89AA25BC8599}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>